<commit_message>
Termino primer entrega (falta metodologia, arreglar detalles y mejorar el repo)
</commit_message>
<xml_diff>
--- a/Informe/Tablas/tabla_base_construida.xlsx
+++ b/Informe/Tablas/tabla_base_construida.xlsx
@@ -101,9 +101,6 @@
     <t>Precio de la Soja</t>
   </si>
   <si>
-    <t>Precio del Maiz</t>
-  </si>
-  <si>
     <t>Precio del Sorgo</t>
   </si>
   <si>
@@ -192,6 +189,9 @@
   </si>
   <si>
     <t>Cuantitativa Continua</t>
+  </si>
+  <si>
+    <t>Precio del Maíz</t>
   </si>
 </sst>
 </file>
@@ -557,10 +557,10 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
@@ -568,76 +568,76 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C2" t="s">
         <v>53</v>
-      </c>
-      <c r="C2" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
@@ -645,10 +645,10 @@
         <v>2</v>
       </c>
       <c r="B9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
@@ -656,10 +656,10 @@
         <v>3</v>
       </c>
       <c r="B10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
@@ -670,7 +670,7 @@
         <v>22</v>
       </c>
       <c r="C11" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
@@ -681,7 +681,7 @@
         <v>23</v>
       </c>
       <c r="C12" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
@@ -692,7 +692,7 @@
         <v>24</v>
       </c>
       <c r="C13" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
@@ -700,10 +700,10 @@
         <v>7</v>
       </c>
       <c r="B14" t="s">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="C14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
@@ -711,10 +711,10 @@
         <v>8</v>
       </c>
       <c r="B15" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C15" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
@@ -722,10 +722,10 @@
         <v>9</v>
       </c>
       <c r="B16" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
@@ -733,10 +733,10 @@
         <v>10</v>
       </c>
       <c r="B17" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C17" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
@@ -744,10 +744,10 @@
         <v>11</v>
       </c>
       <c r="B18" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C18" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
@@ -755,10 +755,10 @@
         <v>12</v>
       </c>
       <c r="B19" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C19" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
@@ -766,10 +766,10 @@
         <v>13</v>
       </c>
       <c r="B20" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C20" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
@@ -777,7 +777,7 @@
         <v>14</v>
       </c>
       <c r="C21" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
@@ -785,10 +785,10 @@
         <v>15</v>
       </c>
       <c r="B22" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C22" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
@@ -796,10 +796,10 @@
         <v>16</v>
       </c>
       <c r="B23" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C23" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
@@ -807,10 +807,10 @@
         <v>17</v>
       </c>
       <c r="B24" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C24" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.35">
@@ -818,10 +818,10 @@
         <v>18</v>
       </c>
       <c r="B25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.35">
@@ -829,7 +829,7 @@
         <v>19</v>
       </c>
       <c r="C26" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.35">
@@ -837,7 +837,7 @@
         <v>20</v>
       </c>
       <c r="C27" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.35">
@@ -845,10 +845,10 @@
         <v>21</v>
       </c>
       <c r="B28" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C28" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Aplicacion (falta sombreado) y Anexo (falta justificar cond y exp q son no estac) casi terminados. Foto antes de cambiar justif imput
</commit_message>
<xml_diff>
--- a/Informe/Tablas/tabla_base_construida.xlsx
+++ b/Informe/Tablas/tabla_base_construida.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="59">
   <si>
     <t>Variable</t>
   </si>
@@ -192,6 +192,15 @@
   </si>
   <si>
     <t>Precio del Maíz</t>
+  </si>
+  <si>
+    <t>Rendimiento de las 30 mayores empresas de EEUU</t>
+  </si>
+  <si>
+    <t>Evolución precio de acciones de empresas tecnológicas</t>
+  </si>
+  <si>
+    <t>Tasa de fondos federales de EEUU</t>
   </si>
 </sst>
 </file>
@@ -776,6 +785,9 @@
       <c r="A21" t="s">
         <v>14</v>
       </c>
+      <c r="B21" t="s">
+        <v>58</v>
+      </c>
       <c r="C21" t="s">
         <v>54</v>
       </c>
@@ -828,6 +840,9 @@
       <c r="A26" t="s">
         <v>19</v>
       </c>
+      <c r="B26" t="s">
+        <v>57</v>
+      </c>
       <c r="C26" t="s">
         <v>54</v>
       </c>
@@ -835,6 +850,9 @@
     <row r="27" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>20</v>
+      </c>
+      <c r="B27" t="s">
+        <v>56</v>
       </c>
       <c r="C27" t="s">
         <v>54</v>

</xml_diff>